<commit_message>
feat: Motor CPE v4.0 — DbfFarmaciaAdapter, TxtGenerator APIFAS, ClientLoader, CpeLogger SQLite, Motor orquestador
</commit_message>
<xml_diff>
--- a/ventas_pos_prueba.xlsx
+++ b/ventas_pos_prueba.xlsx
@@ -579,7 +579,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -676,7 +676,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">

</xml_diff>